<commit_message>
Update SDG output axis and research data
</commit_message>
<xml_diff>
--- a/研究量能統計 2018-2025.xlsx
+++ b/研究量能統計 2018-2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\喬文作業區\線上追蹤平台\研究量能追蹤平台\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C69D0827-378A-4A59-8935-556DFB3731B1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68A9DDBB-CD44-4C2C-A4BC-13C34FF8024D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8556" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">General!$A$1:$W$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">QS!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">THE!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">THE!$A$1:$I$289</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -12749,7 +12749,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1" xr:uid="{80358242-D0A4-423E-A4DF-FFB2194CE0AE}">
+  <autoFilter ref="A1:I289" xr:uid="{80358242-D0A4-423E-A4DF-FFB2194CE0AE}">
     <sortState ref="A2:I289">
       <sortCondition ref="C1"/>
     </sortState>

</xml_diff>